<commit_message>
Add paper draft history and formatted analysis workbook
</commit_message>
<xml_diff>
--- a/results/analysis/main_001_analysis_dataset V0.2.xlsx
+++ b/results/analysis/main_001_analysis_dataset V0.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\3-6-2023\muawia 03-06-2026\Agentic-AI-research\results\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A200335E-1E09-4C08-99B5-6C1A463009D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF98D82-563F-4B49-8135-169AF9B27AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{57F7D5C2-D45C-42EC-B4CA-9E47A6AE5B19}"/>
+    <workbookView xWindow="-23148" yWindow="1056" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{57F7D5C2-D45C-42EC-B4CA-9E47A6AE5B19}"/>
   </bookViews>
   <sheets>
     <sheet name="main_001_analysis_dataset" sheetId="6" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1780" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="438">
   <si>
     <t>run_id</t>
   </si>
@@ -2213,6 +2213,15 @@
   <si>
     <t>Total Runs</t>
   </si>
+  <si>
+    <t>Workflow</t>
+  </si>
+  <si>
+    <t>Planner Executor Improvement over Basic</t>
+  </si>
+  <si>
+    <t>Planner Executor Reviewer Improvement over Basic</t>
+  </si>
 </sst>
 </file>
 
@@ -2222,7 +2231,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2357,8 +2366,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2538,8 +2560,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -2654,6 +2682,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2700,7 +2839,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2740,7 +2879,68 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2787,51 +2987,579 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="48">
+  <dxfs count="70">
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2873,13 +3601,19 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
@@ -2932,6 +3666,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -18643,7 +19389,7 @@
     <dataField name="StdDev of confidence" fld="9" subtotal="stdDev" baseField="3" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="5">
+    <format dxfId="66">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2" selected="0">
@@ -18800,7 +19546,7 @@
     <dataField name="Count of confidence" fld="9" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="3">
+    <format dxfId="67">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4" selected="0">
@@ -19037,7 +19783,7 @@
     <dataField name="StdDev of quality_score" fld="10" subtotal="stdDev" baseField="3" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="34">
+    <format dxfId="69">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19046,7 +19792,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="68">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19083,100 +19829,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3BDF74AC-CC0A-4F7A-A82A-3B8CCA7B753A}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
-  <location ref="D5:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="21">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="22" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="18"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="3" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Average of confidence" fld="9" subtotal="average" baseField="18" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="30">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2ED65D1C-A30A-40CF-A385-248F068BFEE0}" name="PivotTable5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="D23:H28" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="21">
@@ -19254,14 +19906,14 @@
     <dataField name="Average of confidence" fld="9" subtotal="average" baseField="3" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="32">
+    <format dxfId="51">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="50">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19369,6 +20021,100 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3BDF74AC-CC0A-4F7A-A82A-3B8CCA7B753A}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="D5:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="21">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="22" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="18"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="3" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Average of confidence" fld="9" subtotal="average" baseField="18" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="52">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{95A74D01-4A39-4E0D-9F7D-78C3B48524C1}" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="C16:G21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
@@ -19447,7 +20193,7 @@
     <dataField name="Average of confidence" fld="9" subtotal="average" baseField="3" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="28">
+    <format dxfId="48">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19595,7 +20341,7 @@
     <dataField name="Average of confidence" fld="9" subtotal="average" baseField="19" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="29">
+    <format dxfId="49">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19706,30 +20452,30 @@
   </autoFilter>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{4F7162D1-3790-4A9C-9072-26DFB948AD19}" uniqueName="1" name="run_id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{3C0D94D1-A82C-4CF4-9391-DF02DEB32370}" uniqueName="2" name="experiment_id" queryTableFieldId="2" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{3C0D94D1-A82C-4CF4-9391-DF02DEB32370}" uniqueName="2" name="experiment_id" queryTableFieldId="2" dataDxfId="65"/>
     <tableColumn id="3" xr3:uid="{FC4FD114-4FF2-401E-B840-E8E08BC05447}" uniqueName="3" name="task_id" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{3FC0A036-E406-4B1D-AAAF-07982CB5929F}" uniqueName="4" name="workflow_type" queryTableFieldId="4" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{F64A6674-480E-44E5-AD6A-B60679F9A6D6}" uniqueName="5" name="timestamp" queryTableFieldId="5" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{29D68B0E-322F-4C8A-AAD8-035B1C1BFE6E}" uniqueName="6" name="prompt" queryTableFieldId="6" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{7A79A79D-E84E-4EA7-A604-B8A9303184F7}" uniqueName="7" name="output" queryTableFieldId="7" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{688FAF55-DC21-4B4B-8DFB-860A6DAE5C94}" uniqueName="8" name="answer" queryTableFieldId="8" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{3EB6F32C-FC13-47E0-ACAB-31ABC81D446F}" uniqueName="9" name="execution_summary" queryTableFieldId="9" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{3FC0A036-E406-4B1D-AAAF-07982CB5929F}" uniqueName="4" name="workflow_type" queryTableFieldId="4" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{F64A6674-480E-44E5-AD6A-B60679F9A6D6}" uniqueName="5" name="timestamp" queryTableFieldId="5" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{29D68B0E-322F-4C8A-AAD8-035B1C1BFE6E}" uniqueName="6" name="prompt" queryTableFieldId="6" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{7A79A79D-E84E-4EA7-A604-B8A9303184F7}" uniqueName="7" name="output" queryTableFieldId="7" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{688FAF55-DC21-4B4B-8DFB-860A6DAE5C94}" uniqueName="8" name="answer" queryTableFieldId="8" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{3EB6F32C-FC13-47E0-ACAB-31ABC81D446F}" uniqueName="9" name="execution_summary" queryTableFieldId="9" dataDxfId="59"/>
     <tableColumn id="10" xr3:uid="{2AEC909B-9BDA-4D54-96E3-388D29533592}" uniqueName="10" name="confidence" queryTableFieldId="10"/>
     <tableColumn id="11" xr3:uid="{FD182298-DEBB-493C-A8C8-93D40AE13567}" uniqueName="11" name="quality_score" queryTableFieldId="11"/>
     <tableColumn id="12" xr3:uid="{25D0B228-FBAB-4F9E-B575-EC3B6A29C427}" uniqueName="12" name="score" queryTableFieldId="12"/>
     <tableColumn id="13" xr3:uid="{5BD431FF-6410-4D4D-8142-9927364ECBEC}" uniqueName="13" name="duration_sec" queryTableFieldId="13"/>
     <tableColumn id="14" xr3:uid="{A8B4D324-1AA7-47C4-A118-EC65A2B5DB00}" uniqueName="14" name="token_estimate" queryTableFieldId="14"/>
     <tableColumn id="15" xr3:uid="{134EB055-6B5D-40FB-B253-B9F83987C508}" uniqueName="15" name="success" queryTableFieldId="15"/>
-    <tableColumn id="16" xr3:uid="{C42D9C25-8525-408D-90FA-2844A1B50667}" uniqueName="16" name="notes" queryTableFieldId="16" dataDxfId="40"/>
-    <tableColumn id="17" xr3:uid="{C319D253-1672-4B72-8E58-7B4489A4B105}" uniqueName="17" name="reviewer_version" queryTableFieldId="17" dataDxfId="39"/>
-    <tableColumn id="18" xr3:uid="{E82B4081-5BE1-46E1-A169-5F5F84091853}" uniqueName="18" name="real_task_id" queryTableFieldId="18" dataDxfId="38"/>
-    <tableColumn id="19" xr3:uid="{897CC1A7-FBD0-4512-8FB2-15CD91BC7E72}" uniqueName="19" name="category" queryTableFieldId="19" dataDxfId="37">
+    <tableColumn id="16" xr3:uid="{C42D9C25-8525-408D-90FA-2844A1B50667}" uniqueName="16" name="notes" queryTableFieldId="16" dataDxfId="58"/>
+    <tableColumn id="17" xr3:uid="{C319D253-1672-4B72-8E58-7B4489A4B105}" uniqueName="17" name="reviewer_version" queryTableFieldId="17" dataDxfId="57"/>
+    <tableColumn id="18" xr3:uid="{E82B4081-5BE1-46E1-A169-5F5F84091853}" uniqueName="18" name="real_task_id" queryTableFieldId="18" dataDxfId="56"/>
+    <tableColumn id="19" xr3:uid="{897CC1A7-FBD0-4512-8FB2-15CD91BC7E72}" uniqueName="19" name="category" queryTableFieldId="19" dataDxfId="55">
       <calculatedColumnFormula>VLOOKUP(main_001_90runs__2[[#This Row],[prompt]],tasks!B:E,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{8AD98BD3-95E8-47C4-AF92-7FE9804C536D}" uniqueName="20" name="difficulty" queryTableFieldId="20" dataDxfId="36">
+    <tableColumn id="20" xr3:uid="{8AD98BD3-95E8-47C4-AF92-7FE9804C536D}" uniqueName="20" name="difficulty" queryTableFieldId="20" dataDxfId="54">
       <calculatedColumnFormula>VLOOKUP(main_001_90runs__2[[#This Row],[prompt]],tasks!B:E,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{9446655C-2110-43B2-8D39-E8CFB28CF583}" uniqueName="21" name="expected_output" queryTableFieldId="21" dataDxfId="35">
+    <tableColumn id="21" xr3:uid="{9446655C-2110-43B2-8D39-E8CFB28CF583}" uniqueName="21" name="expected_output" queryTableFieldId="21" dataDxfId="53">
       <calculatedColumnFormula>VLOOKUP(main_001_90runs__2[[#This Row],[prompt]],tasks!B:E,4,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -19738,51 +20484,101 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5844FB2E-82F6-42F8-BF1E-9034BA11F61F}" name="Table4" displayName="Table4" ref="C5:D13" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{716C986D-0B58-4F25-BDDA-3CDA15B5F612}" name="Table5" displayName="Table5" ref="G57:I60" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="29" tableBorderDxfId="30" totalsRowBorderDxfId="28">
+  <autoFilter ref="G57:I60" xr:uid="{716C986D-0B58-4F25-BDDA-3CDA15B5F612}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{45A44148-1718-4D40-B68D-E31C248EF02F}" name="Workflow" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{D7143E0E-0D36-408B-9507-9E17F271D932}" name="Average of confidence" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{0E819C8D-2C8A-4020-8B73-0427AA343E63}" name="StdDev of confidence" dataDxfId="25"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F9366993-2B46-4266-8419-992FD0C5D70C}" name="Table6" displayName="Table6" ref="M23:P26" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="22" tableBorderDxfId="23" totalsRowBorderDxfId="21">
+  <autoFilter ref="M23:P26" xr:uid="{F9366993-2B46-4266-8419-992FD0C5D70C}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{FCF27EEB-7BEA-4C34-8AFB-6348A3BCA5CE}" name="Row Labels" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{842B091D-ABF0-4DD9-937C-0533D65FEC34}" name="Coding" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{15266354-7073-4624-AC65-87DEC4DD31B9}" name="Knowledge" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{BA824A2C-13D2-4A16-838F-AB76E4ED3325}" name="Reasoning" dataDxfId="17"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{224961FA-B546-4DE7-8D20-31EA3DDB4407}" name="Table7" displayName="Table7" ref="K17:N20" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
+  <autoFilter ref="K17:N20" xr:uid="{224961FA-B546-4DE7-8D20-31EA3DDB4407}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{91F4001A-739C-443E-8795-7E21A1902377}" name="Row Labels" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{DF04A160-D62B-4F33-9A6A-C41AB72EFF48}" name="easy" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{29CBA7E9-7D4E-4660-89FE-C69EAB6D4BD6}" name="hard" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{D6FCEE01-E98C-4FA2-8352-196F5B0E0CA0}" name="medium" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{5D69EE80-38C5-43CB-9678-847F49099776}" name="Table8" displayName="Table8" ref="H14:J17" totalsRowShown="0" headerRowDxfId="0" dataDxfId="7" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+  <autoFilter ref="H14:J17" xr:uid="{5D69EE80-38C5-43CB-9678-847F49099776}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{89FDD296-035A-4610-A51D-9CCCCCEB6D5A}" name="Metric" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{F8AF7004-5009-4108-A7D2-D8944D7B1B6B}" name="Planner Executor Improvement over Basic" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{748914BE-D9A6-40BE-8D6C-3362758C9D5B}" name="Planner Executor Reviewer Improvement over Basic" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5844FB2E-82F6-42F8-BF1E-9034BA11F61F}" name="Table4" displayName="Table4" ref="C5:D13" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="C5:D13" xr:uid="{5844FB2E-82F6-42F8-BF1E-9034BA11F61F}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{279D2C7F-5E85-49F8-973E-30D6D271E450}" name="Finding" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{98772264-FE01-478F-8BF8-530476C1D303}" name="Result" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{279D2C7F-5E85-49F8-973E-30D6D271E450}" name="Finding" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{98772264-FE01-478F-8BF8-530476C1D303}" name="Result" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{87E4C6D9-89FF-44EE-BA0C-4B066F12A329}" name="main_001_90runs" displayName="main_001_90runs" ref="A1:Q100" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:Q100" xr:uid="{87E4C6D9-89FF-44EE-BA0C-4B066F12A329}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{1601DDC9-6BAD-44C0-9A5C-5A60EAB334D4}" uniqueName="1" name="run_id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{77F976FC-C557-41DF-8BFE-89FC8B8BC07A}" uniqueName="2" name="experiment_id" queryTableFieldId="2" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{77F976FC-C557-41DF-8BFE-89FC8B8BC07A}" uniqueName="2" name="experiment_id" queryTableFieldId="2" dataDxfId="43"/>
     <tableColumn id="3" xr3:uid="{EF24BC62-93C5-4924-88A0-3D706F7724C3}" uniqueName="3" name="task_id" queryTableFieldId="3"/>
-    <tableColumn id="4" xr3:uid="{DE0A40F3-C5FE-4B39-878F-06DFD4EC6147}" uniqueName="4" name="workflow_type" queryTableFieldId="4" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{473401F0-76F0-431B-9920-C76B0F1E56D8}" uniqueName="5" name="timestamp" queryTableFieldId="5" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{5BA58FFB-A745-4AE4-8668-19A3A915A3EB}" uniqueName="6" name="prompt" queryTableFieldId="6" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{EFEEE256-3845-42EC-BC95-822284899B5E}" uniqueName="7" name="output" queryTableFieldId="7" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{94891E91-4BB1-4EAB-813A-4A6FADD4EF88}" uniqueName="8" name="answer" queryTableFieldId="8" dataDxfId="22"/>
-    <tableColumn id="9" xr3:uid="{481D76A0-FBC9-48C6-AF6C-4D63B5002FFC}" uniqueName="9" name="execution_summary" queryTableFieldId="9" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{DE0A40F3-C5FE-4B39-878F-06DFD4EC6147}" uniqueName="4" name="workflow_type" queryTableFieldId="4" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{473401F0-76F0-431B-9920-C76B0F1E56D8}" uniqueName="5" name="timestamp" queryTableFieldId="5" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{5BA58FFB-A745-4AE4-8668-19A3A915A3EB}" uniqueName="6" name="prompt" queryTableFieldId="6" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{EFEEE256-3845-42EC-BC95-822284899B5E}" uniqueName="7" name="output" queryTableFieldId="7" dataDxfId="39"/>
+    <tableColumn id="8" xr3:uid="{94891E91-4BB1-4EAB-813A-4A6FADD4EF88}" uniqueName="8" name="answer" queryTableFieldId="8" dataDxfId="38"/>
+    <tableColumn id="9" xr3:uid="{481D76A0-FBC9-48C6-AF6C-4D63B5002FFC}" uniqueName="9" name="execution_summary" queryTableFieldId="9" dataDxfId="37"/>
     <tableColumn id="10" xr3:uid="{1C55F1EB-5F93-46CE-91B0-D40B791C4DAB}" uniqueName="10" name="confidence" queryTableFieldId="10"/>
     <tableColumn id="11" xr3:uid="{1D423C67-57DE-46E7-A9F9-D3534543F42A}" uniqueName="11" name="quality_score" queryTableFieldId="11"/>
     <tableColumn id="12" xr3:uid="{3FB89599-73DD-4B41-99F0-51B6AE366630}" uniqueName="12" name="score" queryTableFieldId="12"/>
     <tableColumn id="13" xr3:uid="{777E965D-53C2-44B8-A7E5-45A5DCE18480}" uniqueName="13" name="duration_sec" queryTableFieldId="13"/>
     <tableColumn id="14" xr3:uid="{41FD8E6B-2C5E-49E4-A475-C3F0DE35ACFB}" uniqueName="14" name="token_estimate" queryTableFieldId="14"/>
     <tableColumn id="15" xr3:uid="{0069A20F-3F83-4962-8D08-455768B79F34}" uniqueName="15" name="success" queryTableFieldId="15"/>
-    <tableColumn id="16" xr3:uid="{9C9F84B1-97FF-40BF-B721-9459EF544445}" uniqueName="16" name="notes" queryTableFieldId="16" dataDxfId="20"/>
-    <tableColumn id="17" xr3:uid="{0F1832ED-8692-420C-B5F1-844F6AC8FA49}" uniqueName="17" name="reviewer_version" queryTableFieldId="17" dataDxfId="19"/>
+    <tableColumn id="16" xr3:uid="{9C9F84B1-97FF-40BF-B721-9459EF544445}" uniqueName="16" name="notes" queryTableFieldId="16" dataDxfId="36"/>
+    <tableColumn id="17" xr3:uid="{0F1832ED-8692-420C-B5F1-844F6AC8FA49}" uniqueName="17" name="reviewer_version" queryTableFieldId="17" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{55368ADF-F182-4E67-9256-0C633E91E6A6}" name="tasks" displayName="tasks" ref="A1:E33" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E33" xr:uid="{55368ADF-F182-4E67-9256-0C633E91E6A6}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{5C844240-A857-4ABC-81D9-B2ABE1450D53}" uniqueName="1" name="task_id" queryTableFieldId="1"/>
-    <tableColumn id="6" xr3:uid="{5B81FDCB-27B3-4D2E-9F9B-F4FBF4E93770}" uniqueName="6" name="task" queryTableFieldId="6" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{861D80BF-B6F9-4E08-B60F-6DE453C51C3E}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{1FF47BD3-780D-4448-B848-8D6FE6428415}" uniqueName="3" name="difficulty" queryTableFieldId="3" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{DE1E4470-3ADD-487F-84EB-11304B9CAFCB}" uniqueName="5" name="expected_output" queryTableFieldId="5" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{5B81FDCB-27B3-4D2E-9F9B-F4FBF4E93770}" uniqueName="6" name="task" queryTableFieldId="6" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{861D80BF-B6F9-4E08-B60F-6DE453C51C3E}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{1FF47BD3-780D-4448-B848-8D6FE6428415}" uniqueName="3" name="difficulty" queryTableFieldId="3" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{DE1E4470-3ADD-487F-84EB-11304B9CAFCB}" uniqueName="5" name="expected_output" queryTableFieldId="5" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -20086,30 +20882,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A008CD7-1CB8-40CE-96F3-0D1926DE5CBA}">
   <dimension ref="A1:U91"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" customWidth="1"/>
-    <col min="5" max="5" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="68.109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="7.6640625" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" customWidth="1"/>
-    <col min="9" max="9" width="5.33203125" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="68.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="7.7109375" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
+    <col min="9" max="9" width="5.28515625" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" customWidth="1"/>
+    <col min="11" max="11" width="7.7109375" customWidth="1"/>
     <col min="12" max="12" width="6" customWidth="1"/>
-    <col min="13" max="13" width="8.44140625" customWidth="1"/>
-    <col min="14" max="14" width="2.77734375" customWidth="1"/>
-    <col min="15" max="15" width="8.33203125" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" customWidth="1"/>
+    <col min="14" max="14" width="2.7109375" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" customWidth="1"/>
     <col min="17" max="17" width="19" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -20174,7 +20970,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1780574892946</v>
       </c>
@@ -20239,7 +21035,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="3" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1780574903737</v>
       </c>
@@ -20304,7 +21100,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="4" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1780574915175</v>
       </c>
@@ -20372,7 +21168,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1780575855817</v>
       </c>
@@ -20437,7 +21233,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1780575867997</v>
       </c>
@@ -20502,7 +21298,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1780575879320</v>
       </c>
@@ -20570,7 +21366,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1780576994343</v>
       </c>
@@ -20635,7 +21431,7 @@
         <v>Comparison report</v>
       </c>
     </row>
-    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1780577003965</v>
       </c>
@@ -20700,7 +21496,7 @@
         <v>Comparison report</v>
       </c>
     </row>
-    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1780577017923</v>
       </c>
@@ -20768,7 +21564,7 @@
         <v>Comparison report</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1780578566594</v>
       </c>
@@ -20833,7 +21629,7 @@
         <v>Executive summary</v>
       </c>
     </row>
-    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1780578577218</v>
       </c>
@@ -20898,7 +21694,7 @@
         <v>Executive summary</v>
       </c>
     </row>
-    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1780578589961</v>
       </c>
@@ -20966,7 +21762,7 @@
         <v>Executive summary</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1780578618719</v>
       </c>
@@ -21031,7 +21827,7 @@
         <v>Risk assessment</v>
       </c>
     </row>
-    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1780578629992</v>
       </c>
@@ -21096,7 +21892,7 @@
         <v>Risk assessment</v>
       </c>
     </row>
-    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1780578642455</v>
       </c>
@@ -21164,7 +21960,7 @@
         <v>Risk assessment</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1780592134171</v>
       </c>
@@ -21229,7 +22025,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1780592144663</v>
       </c>
@@ -21294,7 +22090,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1780592161109</v>
       </c>
@@ -21362,7 +22158,7 @@
         <v>Structured comparison</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1780592416686</v>
       </c>
@@ -21427,7 +22223,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1780592437302</v>
       </c>
@@ -21492,7 +22288,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1780592453508</v>
       </c>
@@ -21560,7 +22356,7 @@
         <v>Technical explanation</v>
       </c>
     </row>
-    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1780592534321</v>
       </c>
@@ -21625,7 +22421,7 @@
         <v>Metric framework</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1780594284298</v>
       </c>
@@ -21690,7 +22486,7 @@
         <v>Metric framework</v>
       </c>
     </row>
-    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1780592545486</v>
       </c>
@@ -21758,7 +22554,7 @@
         <v>Metric framework</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1780592630484</v>
       </c>
@@ -21823,7 +22619,7 @@
         <v>Analytical report</v>
       </c>
     </row>
-    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1780592643747</v>
       </c>
@@ -21888,7 +22684,7 @@
         <v>Analytical report</v>
       </c>
     </row>
-    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1780592655630</v>
       </c>
@@ -21956,7 +22752,7 @@
         <v>Analytical report</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1780592707411</v>
       </c>
@@ -22021,7 +22817,7 @@
         <v>Architecture recommendation</v>
       </c>
     </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1780592721050</v>
       </c>
@@ -22086,7 +22882,7 @@
         <v>Architecture recommendation</v>
       </c>
     </row>
-    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1780592738156</v>
       </c>
@@ -22154,7 +22950,7 @@
         <v>Architecture recommendation</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1780596118666</v>
       </c>
@@ -22219,7 +23015,7 @@
         <v>Solution recommendation</v>
       </c>
     </row>
-    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1780596135290</v>
       </c>
@@ -22284,7 +23080,7 @@
         <v>Solution recommendation</v>
       </c>
     </row>
-    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1780596152936</v>
       </c>
@@ -22352,7 +23148,7 @@
         <v>Solution recommendation</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1780596953667</v>
       </c>
@@ -22417,7 +23213,7 @@
         <v>Priority classification</v>
       </c>
     </row>
-    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1780596966596</v>
       </c>
@@ -22482,7 +23278,7 @@
         <v>Priority classification</v>
       </c>
     </row>
-    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1780596983555</v>
       </c>
@@ -22550,7 +23346,7 @@
         <v>Priority classification</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1780597606685</v>
       </c>
@@ -22615,7 +23411,7 @@
         <v>Workflow design</v>
       </c>
     </row>
-    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1780597621343</v>
       </c>
@@ -22680,7 +23476,7 @@
         <v>Workflow design</v>
       </c>
     </row>
-    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1780597634783</v>
       </c>
@@ -22748,7 +23544,7 @@
         <v>Workflow design</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1780598933183</v>
       </c>
@@ -22813,7 +23609,7 @@
         <v>Automation recommendations</v>
       </c>
     </row>
-    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1780598947098</v>
       </c>
@@ -22878,7 +23674,7 @@
         <v>Automation recommendations</v>
       </c>
     </row>
-    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1780598961920</v>
       </c>
@@ -22946,7 +23742,7 @@
         <v>Automation recommendations</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1780599009856</v>
       </c>
@@ -23011,7 +23807,7 @@
         <v>Report template</v>
       </c>
     </row>
-    <row r="45" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1780599025011</v>
       </c>
@@ -23076,7 +23872,7 @@
         <v>Report template</v>
       </c>
     </row>
-    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1780599040960</v>
       </c>
@@ -23144,7 +23940,7 @@
         <v>Report template</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1780599513611</v>
       </c>
@@ -23209,7 +24005,7 @@
         <v>Professional response</v>
       </c>
     </row>
-    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1780599526940</v>
       </c>
@@ -23274,7 +24070,7 @@
         <v>Professional response</v>
       </c>
     </row>
-    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>1780599544886</v>
       </c>
@@ -23342,7 +24138,7 @@
         <v>Professional response</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>1780602749112</v>
       </c>
@@ -23407,7 +24203,7 @@
         <v>Theme analysis</v>
       </c>
     </row>
-    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>1780602760115</v>
       </c>
@@ -23472,7 +24268,7 @@
         <v>Theme analysis</v>
       </c>
     </row>
-    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>1780602781195</v>
       </c>
@@ -23540,7 +24336,7 @@
         <v>Theme analysis</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>1780602801867</v>
       </c>
@@ -23605,7 +24401,7 @@
         <v>Status update template</v>
       </c>
     </row>
-    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>1780602822044</v>
       </c>
@@ -23670,7 +24466,7 @@
         <v>Status update template</v>
       </c>
     </row>
-    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>1780602837863</v>
       </c>
@@ -23738,7 +24534,7 @@
         <v>Status update template</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>1780603555118</v>
       </c>
@@ -23803,7 +24599,7 @@
         <v>KPI framework</v>
       </c>
     </row>
-    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>1780603573661</v>
       </c>
@@ -23868,7 +24664,7 @@
         <v>KPI framework</v>
       </c>
     </row>
-    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>1780603608918</v>
       </c>
@@ -23936,7 +24732,7 @@
         <v>KPI framework</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>1780605237361</v>
       </c>
@@ -24001,7 +24797,7 @@
         <v>Disaster recovery strategy</v>
       </c>
     </row>
-    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>1780605256470</v>
       </c>
@@ -24066,7 +24862,7 @@
         <v>Disaster recovery strategy</v>
       </c>
     </row>
-    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>1780605280827</v>
       </c>
@@ -24134,7 +24930,7 @@
         <v>Disaster recovery strategy</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>1780634787426</v>
       </c>
@@ -24199,7 +24995,7 @@
         <v>Python code</v>
       </c>
     </row>
-    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>1780634801127</v>
       </c>
@@ -24264,7 +25060,7 @@
         <v>Python code</v>
       </c>
     </row>
-    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>1780634817329</v>
       </c>
@@ -24332,7 +25128,7 @@
         <v>Python code</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>1780634841289</v>
       </c>
@@ -24397,7 +25193,7 @@
         <v>SQL explanation</v>
       </c>
     </row>
-    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>1780634854354</v>
       </c>
@@ -24462,7 +25258,7 @@
         <v>SQL explanation</v>
       </c>
     </row>
-    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>1780634871339</v>
       </c>
@@ -24530,7 +25326,7 @@
         <v>SQL explanation</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>1780635142656</v>
       </c>
@@ -24595,7 +25391,7 @@
         <v>Code review</v>
       </c>
     </row>
-    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>1780635153411</v>
       </c>
@@ -24660,7 +25456,7 @@
         <v>Code review</v>
       </c>
     </row>
-    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>1780635164675</v>
       </c>
@@ -24728,7 +25524,7 @@
         <v>Code review</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>1780635988192</v>
       </c>
@@ -24793,7 +25589,7 @@
         <v>Integration plan</v>
       </c>
     </row>
-    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>1780636001823</v>
       </c>
@@ -24858,7 +25654,7 @@
         <v>Integration plan</v>
       </c>
     </row>
-    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>1780636024992</v>
       </c>
@@ -24926,7 +25722,7 @@
         <v>Integration plan</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>1780636134963</v>
       </c>
@@ -24991,7 +25787,7 @@
         <v>Pseudocode</v>
       </c>
     </row>
-    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>1780636146258</v>
       </c>
@@ -25056,7 +25852,7 @@
         <v>Pseudocode</v>
       </c>
     </row>
-    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>1780636167836</v>
       </c>
@@ -25124,7 +25920,7 @@
         <v>Pseudocode</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>1780637184549</v>
       </c>
@@ -25189,7 +25985,7 @@
         <v>Debugging report</v>
       </c>
     </row>
-    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>1780637204715</v>
       </c>
@@ -25254,7 +26050,7 @@
         <v>Debugging report</v>
       </c>
     </row>
-    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>1780637219139</v>
       </c>
@@ -25322,7 +26118,7 @@
         <v>Debugging report</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>1780637310429</v>
       </c>
@@ -25387,7 +26183,7 @@
         <v>Database schema</v>
       </c>
     </row>
-    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>1780637334917</v>
       </c>
@@ -25452,7 +26248,7 @@
         <v>Database schema</v>
       </c>
     </row>
-    <row r="82" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>1780637350432</v>
       </c>
@@ -25520,7 +26316,7 @@
         <v>Database schema</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>1780637766559</v>
       </c>
@@ -25585,7 +26381,7 @@
         <v>Test cases</v>
       </c>
     </row>
-    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>1780637782144</v>
       </c>
@@ -25650,7 +26446,7 @@
         <v>Test cases</v>
       </c>
     </row>
-    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>1780637799178</v>
       </c>
@@ -25718,7 +26514,7 @@
         <v>Test cases</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>1780637843444</v>
       </c>
@@ -25783,7 +26579,7 @@
         <v>Implementation guide</v>
       </c>
     </row>
-    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>1780637855951</v>
       </c>
@@ -25848,7 +26644,7 @@
         <v>Implementation guide</v>
       </c>
     </row>
-    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>1780637879625</v>
       </c>
@@ -25916,7 +26712,7 @@
         <v>Implementation guide</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>1780641143921</v>
       </c>
@@ -25981,7 +26777,7 @@
         <v>Workflow design</v>
       </c>
     </row>
-    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>1780641162554</v>
       </c>
@@ -26046,7 +26842,7 @@
         <v>Workflow design</v>
       </c>
     </row>
-    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>1780641179538</v>
       </c>
@@ -26124,16 +26920,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{639820F3-4F6C-43D3-8732-A145F94E6EBF}">
-  <dimension ref="C6:H61"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="C6:I61"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C6" s="6" t="s">
         <v>399</v>
       </c>
@@ -26144,17 +26941,17 @@
         <v>408</v>
       </c>
     </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C7" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C8" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C9" s="7" t="s">
         <v>29</v>
       </c>
@@ -26165,7 +26962,7 @@
         <v>0.10511569980182504</v>
       </c>
     </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C10" s="7" t="s">
         <v>400</v>
       </c>
@@ -26176,12 +26973,12 @@
         <v>0.10511569980182504</v>
       </c>
     </row>
-    <row r="21" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="23" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C23" s="6" t="s">
         <v>399</v>
       </c>
@@ -26201,7 +26998,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="24" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C24" s="7" t="s">
         <v>18</v>
       </c>
@@ -26217,11 +27014,11 @@
       <c r="G24" s="11">
         <v>0.18099342720014833</v>
       </c>
-      <c r="H24" s="17">
+      <c r="H24">
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C25" s="7" t="s">
         <v>24</v>
       </c>
@@ -26237,11 +27034,11 @@
       <c r="G25" s="11">
         <v>2.4625937172205889E-2</v>
       </c>
-      <c r="H25" s="17">
+      <c r="H25">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C26" s="7" t="s">
         <v>29</v>
       </c>
@@ -26257,11 +27054,11 @@
       <c r="G26" s="11">
         <v>2.4869775775559051E-2</v>
       </c>
-      <c r="H26" s="17">
+      <c r="H26">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C27" s="7" t="s">
         <v>400</v>
       </c>
@@ -26277,11 +27074,11 @@
       <c r="G27" s="11">
         <v>0.10638334329365866</v>
       </c>
-      <c r="H27" s="17">
+      <c r="H27">
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C57" s="6" t="s">
         <v>399</v>
       </c>
@@ -26291,8 +27088,17 @@
       <c r="E57" t="s">
         <v>405</v>
       </c>
+      <c r="G57" t="s">
+        <v>435</v>
+      </c>
+      <c r="H57" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="I57" s="18" t="s">
+        <v>405</v>
+      </c>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C58" s="7" t="s">
         <v>18</v>
       </c>
@@ -26302,8 +27108,17 @@
       <c r="E58" s="11">
         <v>0.18099342720014833</v>
       </c>
+      <c r="G58" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H58" s="20">
+        <v>0.94999999999999984</v>
+      </c>
+      <c r="I58" s="21">
+        <v>0.18099342720014833</v>
+      </c>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C59" s="7" t="s">
         <v>24</v>
       </c>
@@ -26313,8 +27128,17 @@
       <c r="E59" s="11">
         <v>2.4625937172205889E-2</v>
       </c>
+      <c r="G59" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="H59" s="20">
+        <v>0.97933333333333317</v>
+      </c>
+      <c r="I59" s="21">
+        <v>2.4625937172205889E-2</v>
+      </c>
     </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C60" s="7" t="s">
         <v>29</v>
       </c>
@@ -26324,8 +27148,17 @@
       <c r="E60" s="11">
         <v>2.4869775775559051E-2</v>
       </c>
+      <c r="G60" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="H60" s="23">
+        <v>0.98566666666666658</v>
+      </c>
+      <c r="I60" s="24">
+        <v>2.4869775775559051E-2</v>
+      </c>
     </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C61" s="7" t="s">
         <v>400</v>
       </c>
@@ -26339,25 +27172,32 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId4"/>
+  <tableParts count="1">
+    <tablePart r:id="rId5"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFE10E64-2552-4C8C-84C7-84D5F8EB1E32}">
-  <dimension ref="D1:H28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="D1:P28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="3" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
@@ -26365,7 +27205,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="5" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D5" s="6" t="s">
         <v>399</v>
       </c>
@@ -26373,7 +27213,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="6" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D6" s="7" t="s">
         <v>378</v>
       </c>
@@ -26381,7 +27221,7 @@
         <v>0.99285714285714288</v>
       </c>
     </row>
-    <row r="7" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D7" s="7" t="s">
         <v>354</v>
       </c>
@@ -26389,7 +27229,7 @@
         <v>0.98266666666666647</v>
       </c>
     </row>
-    <row r="8" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D8" s="7" t="s">
         <v>367</v>
       </c>
@@ -26397,7 +27237,7 @@
         <v>0.94233333333333336</v>
       </c>
     </row>
-    <row r="9" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D9" s="7" t="s">
         <v>400</v>
       </c>
@@ -26405,20 +27245,32 @@
         <v>0.97215909090909169</v>
       </c>
     </row>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D23" s="6" t="s">
         <v>404</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>410</v>
       </c>
+      <c r="M23" s="29" t="s">
+        <v>399</v>
+      </c>
+      <c r="N23" s="30" t="s">
+        <v>378</v>
+      </c>
+      <c r="O23" s="30" t="s">
+        <v>354</v>
+      </c>
+      <c r="P23" s="31" t="s">
+        <v>367</v>
+      </c>
     </row>
-    <row r="24" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D24" s="6" t="s">
         <v>399</v>
       </c>
@@ -26434,8 +27286,20 @@
       <c r="H24" t="s">
         <v>400</v>
       </c>
+      <c r="M24" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="N24" s="25">
+        <v>0.99499999999999988</v>
+      </c>
+      <c r="O24" s="25">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="P24" s="26">
+        <v>0.87999999999999989</v>
+      </c>
     </row>
-    <row r="25" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D25" s="7" t="s">
         <v>18</v>
       </c>
@@ -26451,8 +27315,20 @@
       <c r="H25" s="11">
         <v>0.94999999999999973</v>
       </c>
+      <c r="M25" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="N25" s="25">
+        <v>0.99444444444444435</v>
+      </c>
+      <c r="O25" s="25">
+        <v>0.97999999999999987</v>
+      </c>
+      <c r="P25" s="26">
+        <v>0.96799999999999997</v>
+      </c>
     </row>
-    <row r="26" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D26" s="7" t="s">
         <v>24</v>
       </c>
@@ -26468,8 +27344,20 @@
       <c r="H26" s="11">
         <v>0.98034482758620667</v>
       </c>
+      <c r="M26" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="N26" s="27">
+        <v>0.98888888888888893</v>
+      </c>
+      <c r="O26" s="27">
+        <v>0.99299999999999999</v>
+      </c>
+      <c r="P26" s="28">
+        <v>0.97899999999999987</v>
+      </c>
     </row>
-    <row r="27" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D27" s="7" t="s">
         <v>29</v>
       </c>
@@ -26486,7 +27374,7 @@
         <v>0.98689655172413793</v>
       </c>
     </row>
-    <row r="28" spans="4:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D28" s="7" t="s">
         <v>400</v>
       </c>
@@ -26506,25 +27394,30 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA1E3820-6423-42EB-9B04-266382C691EF}">
-  <dimension ref="C1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="C1:N21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
@@ -26532,7 +27425,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4" s="6" t="s">
         <v>399</v>
       </c>
@@ -26540,7 +27433,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>355</v>
       </c>
@@ -26548,7 +27441,7 @@
         <v>0.98476190476190462</v>
       </c>
     </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" s="7" t="s">
         <v>362</v>
       </c>
@@ -26556,7 +27449,7 @@
         <v>0.9526470588235294</v>
       </c>
     </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" s="7" t="s">
         <v>359</v>
       </c>
@@ -26564,7 +27457,7 @@
         <v>0.98424242424242414</v>
       </c>
     </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" s="7" t="s">
         <v>400</v>
       </c>
@@ -26572,12 +27465,12 @@
         <v>0.97215909090909125</v>
       </c>
     </row>
-    <row r="14" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="16" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C16" s="6" t="s">
         <v>404</v>
       </c>
@@ -26585,7 +27478,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C17" s="6" t="s">
         <v>399</v>
       </c>
@@ -26601,8 +27494,20 @@
       <c r="G17" t="s">
         <v>400</v>
       </c>
+      <c r="K17" s="29" t="s">
+        <v>399</v>
+      </c>
+      <c r="L17" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="M17" s="30" t="s">
+        <v>362</v>
+      </c>
+      <c r="N17" s="31" t="s">
+        <v>359</v>
+      </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C18" s="7" t="s">
         <v>18</v>
       </c>
@@ -26618,8 +27523,20 @@
       <c r="G18" s="12">
         <v>0.94999999999999984</v>
       </c>
+      <c r="K18" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" s="32">
+        <v>0.98571428571428577</v>
+      </c>
+      <c r="M18" s="32">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="N18" s="33">
+        <v>0.98636363636363644</v>
+      </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C19" s="7" t="s">
         <v>24</v>
       </c>
@@ -26635,8 +27552,20 @@
       <c r="G19" s="12">
         <v>0.98034482758620678</v>
       </c>
+      <c r="K19" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="L19" s="32">
+        <v>0.97857142857142865</v>
+      </c>
+      <c r="M19" s="32">
+        <v>0.98000000000000009</v>
+      </c>
+      <c r="N19" s="33">
+        <v>0.98181818181818192</v>
+      </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C20" s="7" t="s">
         <v>29</v>
       </c>
@@ -26652,8 +27581,20 @@
       <c r="G20" s="12">
         <v>0.98689655172413782</v>
       </c>
+      <c r="K20" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="L20" s="34">
+        <v>0.99</v>
+      </c>
+      <c r="M20" s="34">
+        <v>0.98727272727272719</v>
+      </c>
+      <c r="N20" s="35">
+        <v>0.9845454545454545</v>
+      </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C21" s="7" t="s">
         <v>400</v>
       </c>
@@ -26673,23 +27614,28 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5746E5EA-0848-4F15-B029-8A8B6256BF12}">
-  <dimension ref="C4:H16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="C4:J17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C4" s="9" t="s">
         <v>413</v>
       </c>
@@ -26709,7 +27655,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="5" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C5" s="10" t="s">
         <v>414</v>
       </c>
@@ -26731,7 +27677,7 @@
         <v>3.8947368421052668E-2</v>
       </c>
     </row>
-    <row r="6" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:10" ht="30" x14ac:dyDescent="0.25">
       <c r="C6" s="10" t="s">
         <v>367</v>
       </c>
@@ -26753,7 +27699,7 @@
         <v>0.11249999999999998</v>
       </c>
     </row>
-    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:10" ht="30" x14ac:dyDescent="0.25">
       <c r="C7" s="10" t="s">
         <v>415</v>
       </c>
@@ -26775,12 +27721,12 @@
         <v>0.10156249999999996</v>
       </c>
     </row>
-    <row r="12" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="13" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C13" s="9" t="s">
         <v>413</v>
       </c>
@@ -26791,7 +27737,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="14" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C14" s="10" t="s">
         <v>414</v>
       </c>
@@ -26801,8 +27747,17 @@
       <c r="E14" s="15">
         <v>3.8947368421052668E-2</v>
       </c>
+      <c r="H14" s="36" t="s">
+        <v>413</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>436</v>
+      </c>
+      <c r="J14" s="38" t="s">
+        <v>437</v>
+      </c>
     </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:10" ht="30" x14ac:dyDescent="0.25">
       <c r="C15" s="10" t="s">
         <v>367</v>
       </c>
@@ -26812,8 +27767,17 @@
       <c r="E15" s="15">
         <v>0.11249999999999998</v>
       </c>
+      <c r="H15" s="39" t="s">
+        <v>414</v>
+      </c>
+      <c r="I15" s="40">
+        <v>3.1578947368421081E-2</v>
+      </c>
+      <c r="J15" s="41">
+        <v>3.8947368421052668E-2</v>
+      </c>
     </row>
-    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:10" ht="30" x14ac:dyDescent="0.25">
       <c r="C16" s="10" t="s">
         <v>415</v>
       </c>
@@ -26821,25 +27785,48 @@
         <v>9.3749999999999958E-2</v>
       </c>
       <c r="E16" s="15">
+        <v>0.10156249999999996</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>367</v>
+      </c>
+      <c r="I16" s="40">
+        <v>9.9999999999999964E-2</v>
+      </c>
+      <c r="J16" s="41">
+        <v>0.11249999999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H17" s="42" t="s">
+        <v>415</v>
+      </c>
+      <c r="I17" s="43">
+        <v>9.3749999999999958E-2</v>
+      </c>
+      <c r="J17" s="44">
         <v>0.10156249999999996</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{916D2460-9C81-4E69-BBD9-6862E72ABD3C}">
   <dimension ref="C5:D13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="25.6640625" customWidth="1"/>
-    <col min="4" max="4" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>421</v>
       </c>
@@ -26847,7 +27834,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6" s="7" t="s">
         <v>423</v>
       </c>
@@ -26855,7 +27842,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7" s="7" t="s">
         <v>425</v>
       </c>
@@ -26863,7 +27850,7 @@
         <v>0.98699999999999999</v>
       </c>
     </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8" s="7" t="s">
         <v>426</v>
       </c>
@@ -26871,7 +27858,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9" s="7" t="s">
         <v>428</v>
       </c>
@@ -26879,7 +27866,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10" s="7" t="s">
         <v>430</v>
       </c>
@@ -26887,7 +27874,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C11" s="7" t="s">
         <v>432</v>
       </c>
@@ -26895,7 +27882,7 @@
         <v>0.1016</v>
       </c>
     </row>
-    <row r="12" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C12" s="7" t="s">
         <v>433</v>
       </c>
@@ -26903,7 +27890,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C13" s="7" t="s">
         <v>434</v>
       </c>
@@ -26922,26 +27909,26 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA1FA29-B426-4FCB-9BDA-E2136C3EC938}">
   <dimension ref="A1:Q100"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="80.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="80.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="81.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="36" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -26994,7 +27981,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1780564163884</v>
       </c>
@@ -27044,7 +28031,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1780564209381</v>
       </c>
@@ -27094,7 +28081,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1780564226884</v>
       </c>
@@ -27147,7 +28134,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1780564271744</v>
       </c>
@@ -27197,7 +28184,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1780564325613</v>
       </c>
@@ -27247,7 +28234,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1780564342875</v>
       </c>
@@ -27300,7 +28287,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1780564379837</v>
       </c>
@@ -27350,7 +28337,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1780564398865</v>
       </c>
@@ -27400,7 +28387,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1780564419517</v>
       </c>
@@ -27453,7 +28440,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1780574892946</v>
       </c>
@@ -27503,7 +28490,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1780574903737</v>
       </c>
@@ -27553,7 +28540,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1780574915175</v>
       </c>
@@ -27606,7 +28593,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1780575855817</v>
       </c>
@@ -27656,7 +28643,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1780575867997</v>
       </c>
@@ -27706,7 +28693,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1780575879320</v>
       </c>
@@ -27759,7 +28746,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1780576994343</v>
       </c>
@@ -27809,7 +28796,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1780577003965</v>
       </c>
@@ -27859,7 +28846,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1780577017923</v>
       </c>
@@ -27912,7 +28899,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1780578566594</v>
       </c>
@@ -27962,7 +28949,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1780578577218</v>
       </c>
@@ -28012,7 +28999,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1780578589961</v>
       </c>
@@ -28065,7 +29052,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1780578618719</v>
       </c>
@@ -28115,7 +29102,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1780578629992</v>
       </c>
@@ -28165,7 +29152,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1780578642455</v>
       </c>
@@ -28218,7 +29205,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1780592134171</v>
       </c>
@@ -28268,7 +29255,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1780592144663</v>
       </c>
@@ -28318,7 +29305,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1780592161109</v>
       </c>
@@ -28371,7 +29358,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1780592416686</v>
       </c>
@@ -28421,7 +29408,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1780592437302</v>
       </c>
@@ -28471,7 +29458,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1780592453508</v>
       </c>
@@ -28524,7 +29511,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>1780592534321</v>
       </c>
@@ -28574,7 +29561,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>1780592545486</v>
       </c>
@@ -28627,7 +29614,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>1780592630484</v>
       </c>
@@ -28677,7 +29664,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1780592643747</v>
       </c>
@@ -28727,7 +29714,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1780592655630</v>
       </c>
@@ -28780,7 +29767,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1780592707411</v>
       </c>
@@ -28830,7 +29817,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1780592721050</v>
       </c>
@@ -28880,7 +29867,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1780592738156</v>
       </c>
@@ -28933,7 +29920,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1780594284298</v>
       </c>
@@ -28983,7 +29970,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1780596118666</v>
       </c>
@@ -29033,7 +30020,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1780596135290</v>
       </c>
@@ -29083,7 +30070,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1780596152936</v>
       </c>
@@ -29136,7 +30123,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1780596953667</v>
       </c>
@@ -29186,7 +30173,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1780596966596</v>
       </c>
@@ -29236,7 +30223,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1780596983555</v>
       </c>
@@ -29289,7 +30276,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1780597606685</v>
       </c>
@@ -29339,7 +30326,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1780597621343</v>
       </c>
@@ -29389,7 +30376,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>1780597634783</v>
       </c>
@@ -29442,7 +30429,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>1780598933183</v>
       </c>
@@ -29492,7 +30479,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>1780598947098</v>
       </c>
@@ -29542,7 +30529,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>1780598961920</v>
       </c>
@@ -29595,7 +30582,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>1780599009856</v>
       </c>
@@ -29645,7 +30632,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>1780599025011</v>
       </c>
@@ -29695,7 +30682,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>1780599040960</v>
       </c>
@@ -29748,7 +30735,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>1780599513611</v>
       </c>
@@ -29798,7 +30785,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>1780599526940</v>
       </c>
@@ -29848,7 +30835,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>1780599544886</v>
       </c>
@@ -29901,7 +30888,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>1780602749112</v>
       </c>
@@ -29951,7 +30938,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>1780602760115</v>
       </c>
@@ -30001,7 +30988,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>1780602781195</v>
       </c>
@@ -30054,7 +31041,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>1780602801867</v>
       </c>
@@ -30104,7 +31091,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>1780602822044</v>
       </c>
@@ -30154,7 +31141,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>1780602837863</v>
       </c>
@@ -30207,7 +31194,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>1780603555118</v>
       </c>
@@ -30257,7 +31244,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>1780603573661</v>
       </c>
@@ -30307,7 +31294,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>1780603608918</v>
       </c>
@@ -30360,7 +31347,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>1780605237361</v>
       </c>
@@ -30410,7 +31397,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>1780605256470</v>
       </c>
@@ -30460,7 +31447,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>1780605280827</v>
       </c>
@@ -30513,7 +31500,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>1780634787426</v>
       </c>
@@ -30563,7 +31550,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>1780634801127</v>
       </c>
@@ -30613,7 +31600,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>1780634817329</v>
       </c>
@@ -30666,7 +31653,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>1780634841289</v>
       </c>
@@ -30716,7 +31703,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>1780634854354</v>
       </c>
@@ -30766,7 +31753,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>1780634871339</v>
       </c>
@@ -30819,7 +31806,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>1780635142656</v>
       </c>
@@ -30869,7 +31856,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>1780635153411</v>
       </c>
@@ -30919,7 +31906,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>1780635164675</v>
       </c>
@@ -30972,7 +31959,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>1780635988192</v>
       </c>
@@ -31022,7 +32009,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>1780636001823</v>
       </c>
@@ -31072,7 +32059,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>1780636024992</v>
       </c>
@@ -31125,7 +32112,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>1780636134963</v>
       </c>
@@ -31175,7 +32162,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>1780636146258</v>
       </c>
@@ -31225,7 +32212,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>1780636167836</v>
       </c>
@@ -31278,7 +32265,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>1780637184549</v>
       </c>
@@ -31328,7 +32315,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>1780637204715</v>
       </c>
@@ -31378,7 +32365,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>1780637219139</v>
       </c>
@@ -31431,7 +32418,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>1780637310429</v>
       </c>
@@ -31481,7 +32468,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>1780637334917</v>
       </c>
@@ -31531,7 +32518,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>1780637350432</v>
       </c>
@@ -31584,7 +32571,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>1780637766559</v>
       </c>
@@ -31634,7 +32621,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>1780637782144</v>
       </c>
@@ -31684,7 +32671,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>1780637799178</v>
       </c>
@@ -31737,7 +32724,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>1780637843444</v>
       </c>
@@ -31787,7 +32774,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>1780637855951</v>
       </c>
@@ -31837,7 +32824,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>1780637879625</v>
       </c>
@@ -31890,7 +32877,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>1780641143921</v>
       </c>
@@ -31940,7 +32927,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>1780641162554</v>
       </c>
@@ -31990,7 +32977,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>1780641179538</v>
       </c>
@@ -32054,16 +33041,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CF2475E-08D1-44A3-B359-2B972CFA1D76}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="72.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -32080,7 +33067,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -32097,7 +33084,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -32114,7 +33101,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -32131,7 +33118,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -32148,7 +33135,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -32165,7 +33152,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -32182,7 +33169,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -32199,7 +33186,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -32216,7 +33203,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -32233,7 +33220,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -32250,7 +33237,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>366</v>
       </c>
@@ -32264,7 +33251,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -32281,7 +33268,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -32298,7 +33285,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -32315,7 +33302,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -32332,7 +33319,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -32349,7 +33336,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -32366,7 +33353,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -32383,7 +33370,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -32400,7 +33387,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -32417,7 +33404,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -32434,7 +33421,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
         <v>366</v>
       </c>
@@ -32448,7 +33435,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>21</v>
       </c>
@@ -32465,7 +33452,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>22</v>
       </c>
@@ -32482,7 +33469,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -32499,7 +33486,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -32516,7 +33503,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -32533,7 +33520,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
@@ -32550,7 +33537,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
@@ -32567,7 +33554,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
@@ -32584,7 +33571,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
@@ -32601,7 +33588,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>

</xml_diff>